<commit_message>
feat(APS): add labs, others, readme, vivado basics
</commit_message>
<xml_diff>
--- a/.pic/Labs/lab_05_decoder/rv32i_summary.xlsx
+++ b/.pic/Labs/lab_05_decoder/rv32i_summary.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\voult\Desktop\APS-reborn\.pic\Labs\lab_05_decoder\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA97E5B9-6102-46D4-A302-BF886277C454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{EB09394A-D6B3-4632-AD26-E6834047279C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30936" windowHeight="17496"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,27 +29,9 @@
     <t>Instr</t>
   </si>
   <si>
-    <t>Название</t>
-  </si>
-  <si>
-    <t>Функция</t>
-  </si>
-  <si>
-    <t>Описание</t>
-  </si>
-  <si>
-    <t>Формат</t>
-  </si>
-  <si>
-    <t>Пример использования</t>
-  </si>
-  <si>
     <t>add</t>
   </si>
   <si>
-    <t>Сложение</t>
-  </si>
-  <si>
     <t>rd = rs1 + rs2</t>
   </si>
   <si>
@@ -71,9 +47,6 @@
     <t>sub</t>
   </si>
   <si>
-    <t>Вычитание</t>
-  </si>
-  <si>
     <t>rd = rs1 – rs2</t>
   </si>
   <si>
@@ -116,9 +89,6 @@
     <t>sll</t>
   </si>
   <si>
-    <t>Логический сдвиг влево</t>
-  </si>
-  <si>
     <t>rd = rs1 &lt;&lt; rs2</t>
   </si>
   <si>
@@ -128,9 +98,6 @@
     <t>srl</t>
   </si>
   <si>
-    <t>Логический сдвиг вправо</t>
-  </si>
-  <si>
     <t>rd = rs1 &gt;&gt; rs2</t>
   </si>
   <si>
@@ -140,18 +107,12 @@
     <t>sra</t>
   </si>
   <si>
-    <t>Арифметический сдвиг вправо</t>
-  </si>
-  <si>
     <t>rd = rs1 &gt;&gt;&gt; rs2</t>
   </si>
   <si>
     <t>slt</t>
   </si>
   <si>
-    <t>Результат сравнения A &lt; B</t>
-  </si>
-  <si>
     <t>rd = (rs1 &lt; rs2) ? 1 : 0</t>
   </si>
   <si>
@@ -161,18 +122,12 @@
     <t>sltu</t>
   </si>
   <si>
-    <t>Беззнаковое сравнение A &lt; B</t>
-  </si>
-  <si>
     <t>0x3</t>
   </si>
   <si>
     <t>addi</t>
   </si>
   <si>
-    <t>Сложение с константой</t>
-  </si>
-  <si>
     <t>rd = rs1 + imm</t>
   </si>
   <si>
@@ -230,54 +185,36 @@
     <t>lb</t>
   </si>
   <si>
-    <t>Загрузить байт из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][7:0])</t>
   </si>
   <si>
     <t>lh</t>
   </si>
   <si>
-    <t>Загрузить полуслово из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][15:0])</t>
   </si>
   <si>
     <t>lw</t>
   </si>
   <si>
-    <t>Загрузить слово из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][31:0])</t>
   </si>
   <si>
     <t>lbu</t>
   </si>
   <si>
-    <t>Загрузить беззнаковый байт из памяти</t>
-  </si>
-  <si>
     <t>rd = Mem[rs1 + imm][7:0]</t>
   </si>
   <si>
     <t>lhu</t>
   </si>
   <si>
-    <t>Загрузить беззнаковое полуслово из памяти</t>
-  </si>
-  <si>
     <t>rd = Mem[rs1 + imm][15:0]</t>
   </si>
   <si>
     <t>sb</t>
   </si>
   <si>
-    <t>Сохранить байт в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][7:0] = rs2[7:0]</t>
   </si>
   <si>
@@ -287,27 +224,18 @@
     <t>sh</t>
   </si>
   <si>
-    <t>Сохранить полуслово в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][15:0] = rs2[15:0]</t>
   </si>
   <si>
     <t>sw</t>
   </si>
   <si>
-    <t>Сохранить слово в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][31:0] = rs2[31:0]</t>
   </si>
   <si>
     <t>beq</t>
   </si>
   <si>
-    <t>Перейти, если A == B</t>
-  </si>
-  <si>
     <t>if (rs1 == rs2) PC += imm</t>
   </si>
   <si>
@@ -317,48 +245,30 @@
     <t>bne</t>
   </si>
   <si>
-    <t>Перейти, если A != B</t>
-  </si>
-  <si>
     <t>if (rs1 != rs2) PC += imm</t>
   </si>
   <si>
     <t>blt</t>
   </si>
   <si>
-    <t>Перейти, если A &lt; B</t>
-  </si>
-  <si>
     <t>if (rs1 &lt; rs2) PC += imm</t>
   </si>
   <si>
     <t>bge</t>
   </si>
   <si>
-    <t>Перейти, если A &gt;= B</t>
-  </si>
-  <si>
     <t>if (rs1 &gt;= rs2) PC += imm</t>
   </si>
   <si>
     <t>bltu</t>
   </si>
   <si>
-    <t>Перейти, если A &lt; B беззнаковое</t>
-  </si>
-  <si>
     <t>bgeu</t>
   </si>
   <si>
-    <t>Перейти, если A &gt;= B беззнаковое</t>
-  </si>
-  <si>
     <t>jal</t>
   </si>
   <si>
-    <t>Переход с сохранением адреса возврата</t>
-  </si>
-  <si>
     <t>rd = PC + 4; PC += imm</t>
   </si>
   <si>
@@ -368,18 +278,12 @@
     <t>jalr</t>
   </si>
   <si>
-    <t>Переход по регистру с сохранением адреса возврата</t>
-  </si>
-  <si>
     <t>rd = PC + 4; PC = rs1 + imm</t>
   </si>
   <si>
     <t>lui</t>
   </si>
   <si>
-    <t>Загрузить константу в сдвинутую на 12</t>
-  </si>
-  <si>
     <t>rd = imm &lt;&lt; 12</t>
   </si>
   <si>
@@ -389,31 +293,19 @@
     <t>auipc</t>
   </si>
   <si>
-    <t>Сохранить счетчик команд в сумме с константой &lt;&lt; 12</t>
-  </si>
-  <si>
     <t>rd = PC + (imm &lt;&lt; 12)</t>
   </si>
   <si>
     <t>ecall</t>
   </si>
   <si>
-    <t>Передача управления операционной системе</t>
-  </si>
-  <si>
     <t>ebreak</t>
   </si>
   <si>
-    <t>Передача управления отладчику</t>
-  </si>
-  <si>
     <t>fence</t>
   </si>
   <si>
     <t>FENCE</t>
-  </si>
-  <si>
-    <t>Синхронизация инструкций с потоками данных</t>
   </si>
   <si>
     <r>
@@ -2616,22 +2508,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Воспринимать как </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cascadia Code SemiBold"/>
-        <family val="3"/>
-        <charset val="204"/>
-      </rPr>
-      <t>nop</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>E</t>
     </r>
     <r>
@@ -3587,58 +3463,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Записать в регистровый файл значение </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">-регистра.
-Обновить значение </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-регистра в соответствии с вызываемой инструкцией (см. описание).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">csrop </t>
     </r>
     <r>
@@ -3710,9 +3534,6 @@
     </r>
   </si>
   <si>
-    <t>Возврат управления от обработчика прерывания/исключения</t>
-  </si>
-  <si>
     <t>1110011</t>
   </si>
   <si>
@@ -3867,24 +3688,6 @@
   </si>
   <si>
     <t>illegal_instr = 1</t>
-  </si>
-  <si>
-    <t>Побитовое И</t>
-  </si>
-  <si>
-    <t>Побитовое ИЛИ</t>
-  </si>
-  <si>
-    <t>Побитовое Исключающее ИЛИ</t>
-  </si>
-  <si>
-    <t>Побитовое Исключающее ИЛИ с константой</t>
-  </si>
-  <si>
-    <t>Побитовое ИЛИ с константой</t>
-  </si>
-  <si>
-    <t>Побитовое И с константой</t>
   </si>
   <si>
     <r>
@@ -3947,13 +3750,143 @@
       </rPr>
       <t>**</t>
     </r>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>Usage example</t>
+  </si>
+  <si>
+    <t>Addition</t>
+  </si>
+  <si>
+    <t>Subtraction</t>
+  </si>
+  <si>
+    <t>Bitwise exclusive OR</t>
+  </si>
+  <si>
+    <t>Bitwise OR</t>
+  </si>
+  <si>
+    <t>Bitwise AND</t>
+  </si>
+  <si>
+    <t>Logical left shift</t>
+  </si>
+  <si>
+    <t>Logical right shift</t>
+  </si>
+  <si>
+    <t>Arithmetic right shift</t>
+  </si>
+  <si>
+    <t>Result of comparison A &lt; B</t>
+  </si>
+  <si>
+    <t>Unsigned comparison A &lt; B</t>
+  </si>
+  <si>
+    <t>Addition with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise exclusive OR with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise OR with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise AND with a constant</t>
+  </si>
+  <si>
+    <t>Load byte from memory</t>
+  </si>
+  <si>
+    <t>Load halfword from memory</t>
+  </si>
+  <si>
+    <t>Load word from memory</t>
+  </si>
+  <si>
+    <t>Load unsigned byte from memory</t>
+  </si>
+  <si>
+    <t>Load unsigned halfword from memory</t>
+  </si>
+  <si>
+    <t>Store byte to memory</t>
+  </si>
+  <si>
+    <t>Store halfword to memory</t>
+  </si>
+  <si>
+    <t>Store word to memory</t>
+  </si>
+  <si>
+    <t>Branch if A == B</t>
+  </si>
+  <si>
+    <t>Branch if A != B</t>
+  </si>
+  <si>
+    <t>Branch if A &lt; B</t>
+  </si>
+  <si>
+    <t>Branch if A &gt;= B</t>
+  </si>
+  <si>
+    <t>Branch if A &lt; B, unsigned</t>
+  </si>
+  <si>
+    <t>Branch if A &gt;= B, unsigned</t>
+  </si>
+  <si>
+    <t>Jump saving the return address</t>
+  </si>
+  <si>
+    <t>Register jump saving the return address</t>
+  </si>
+  <si>
+    <t>Load a constant shifted left by 12</t>
+  </si>
+  <si>
+    <t>Save the program counter summed with a constant &lt;&lt; 12</t>
+  </si>
+  <si>
+    <t>Synchronization of instructions with data streams</t>
+  </si>
+  <si>
+    <t>Treat as nop</t>
+  </si>
+  <si>
+    <t>Transfer control to the operating system</t>
+  </si>
+  <si>
+    <t>Transfer control to the debugger</t>
+  </si>
+  <si>
+    <t>Return of control from an interrupt/exception handler</t>
+  </si>
+  <si>
+    <t>Write the value of the CS register to the register file.
+Update the value of the CS register according to the invoked instruction (see description).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4070,14 +4003,6 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color rgb="FF000000"/>
-      <name val="Cascadia Code SemiBold"/>
-      <family val="3"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
       <color rgb="FF4472C4"/>
       <name val="Code Saver"/>
       <family val="3"/>
@@ -4538,34 +4463,55 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4582,27 +4528,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4915,1170 +4840,1191 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4B31E3-B287-4359-8B24-03B2324659CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N48"/>
-  <sheetFormatPr defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="21.9" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="87.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="14.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="87.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="B2" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="E2" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F2" s="67" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="I1" s="27" t="s">
+      <c r="H2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+    <row r="3" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="B3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="E3" s="70"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="65" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="68" t="s">
-        <v>186</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="B4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="E4" s="70"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="H4" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+    <row r="5" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="C5" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="66"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="2" t="s">
+      <c r="E5" s="70"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="H5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I5" s="30" t="s">
+        <v>95</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+    <row r="6" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="66"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="2" t="s">
+      <c r="C6" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="E6" s="70"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="66"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="30" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="66"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I6" s="31"/>
     </row>
-    <row r="7" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="21.9" customHeight="1">
       <c r="A7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="70"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="70"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="66"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="32" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="66"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" s="32" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="66"/>
-      <c r="F9" s="69"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="68"/>
       <c r="G9" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I9" s="31"/>
     </row>
-    <row r="10" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="21.9" customHeight="1">
       <c r="A10" s="8" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>39</v>
+        <v>208</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="66"/>
-      <c r="F10" s="69"/>
+        <v>29</v>
+      </c>
+      <c r="E10" s="70"/>
+      <c r="F10" s="68"/>
       <c r="G10" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I10" s="31"/>
     </row>
-    <row r="11" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A11" s="8" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>43</v>
+        <v>209</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="67"/>
-      <c r="F11" s="70"/>
+        <v>29</v>
+      </c>
+      <c r="E11" s="78"/>
+      <c r="F11" s="79"/>
       <c r="G11" s="2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I11" s="33"/>
     </row>
-    <row r="12" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="21.9" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>46</v>
+        <v>210</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="72" t="s">
-        <v>187</v>
+        <v>34</v>
+      </c>
+      <c r="E12" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="80" t="s">
+        <v>152</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" s="65" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H12" s="69" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="21.9" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>232</v>
+        <v>211</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="66"/>
-      <c r="F13" s="69"/>
+        <v>38</v>
+      </c>
+      <c r="E13" s="70"/>
+      <c r="F13" s="68"/>
       <c r="G13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="66"/>
+        <v>11</v>
+      </c>
+      <c r="H13" s="70"/>
       <c r="I13" s="31"/>
     </row>
-    <row r="14" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="21.9" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>142</v>
+        <v>108</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>233</v>
+        <v>212</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="66"/>
-      <c r="F14" s="69"/>
+        <v>40</v>
+      </c>
+      <c r="E14" s="70"/>
+      <c r="F14" s="68"/>
       <c r="G14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="70"/>
+      <c r="I14" s="34" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A15" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="70"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="70"/>
+    </row>
+    <row r="16" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A16" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="F16" s="68"/>
+      <c r="G16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="66"/>
-      <c r="I14" s="34" t="s">
-        <v>140</v>
+      <c r="H16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="66"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="66"/>
+    <row r="17" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A17" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="82"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I17" s="32" t="s">
+        <v>111</v>
+      </c>
     </row>
-    <row r="16" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E16" s="74" t="s">
-        <v>235</v>
-      </c>
-      <c r="F16" s="69"/>
-      <c r="G16" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" s="32" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="75"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" s="32" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="21.9" customHeight="1">
       <c r="A18" s="22" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>148</v>
+        <v>114</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>36</v>
+        <v>207</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="76"/>
-      <c r="F18" s="69"/>
+        <v>48</v>
+      </c>
+      <c r="E18" s="83"/>
+      <c r="F18" s="68"/>
       <c r="G18" s="5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I18" s="31"/>
     </row>
-    <row r="19" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="21.9" customHeight="1">
       <c r="A19" s="8" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>149</v>
+        <v>115</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>39</v>
+        <v>208</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="F19" s="69"/>
+        <v>50</v>
+      </c>
+      <c r="E19" s="84" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="68"/>
       <c r="G19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H19" s="79" t="s">
-        <v>49</v>
+        <v>30</v>
+      </c>
+      <c r="H19" s="86" t="s">
+        <v>36</v>
       </c>
       <c r="I19" s="31"/>
     </row>
-    <row r="20" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A20" s="8" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>43</v>
+        <v>209</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="78"/>
+        <v>50</v>
+      </c>
+      <c r="E20" s="85"/>
       <c r="F20" s="73"/>
       <c r="G20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" s="67"/>
+        <v>32</v>
+      </c>
+      <c r="H20" s="78"/>
       <c r="I20" s="33"/>
     </row>
-    <row r="21" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="21.9" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>66</v>
+        <v>214</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="F21" s="68" t="s">
-        <v>188</v>
+        <v>53</v>
+      </c>
+      <c r="E21" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="67" t="s">
+        <v>153</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H21" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H21" s="77" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="21.9" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="66"/>
-      <c r="F22" s="69"/>
+        <v>55</v>
+      </c>
+      <c r="E22" s="70"/>
+      <c r="F22" s="68"/>
       <c r="G22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="70"/>
+      <c r="I22" s="34" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A23" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="70"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H22" s="66"/>
-      <c r="I22" s="34" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>154</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="66"/>
-      <c r="F23" s="69"/>
-      <c r="G23" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H23" s="66"/>
+      <c r="H23" s="70"/>
       <c r="I23" s="31"/>
     </row>
-    <row r="24" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="21.9" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>156</v>
+        <v>122</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>75</v>
+        <v>217</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="E24" s="66"/>
-      <c r="F24" s="69"/>
+        <v>59</v>
+      </c>
+      <c r="E24" s="70"/>
+      <c r="F24" s="68"/>
       <c r="G24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H24" s="66"/>
+        <v>11</v>
+      </c>
+      <c r="H24" s="70"/>
       <c r="I24" s="32" t="s">
-        <v>155</v>
+        <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A25" s="8" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>157</v>
+        <v>123</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>78</v>
+        <v>218</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E25" s="67"/>
+        <v>61</v>
+      </c>
+      <c r="E25" s="78"/>
       <c r="F25" s="73"/>
       <c r="G25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H25" s="67"/>
+        <v>25</v>
+      </c>
+      <c r="H25" s="78"/>
       <c r="I25" s="33"/>
     </row>
-    <row r="26" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" ht="21.9" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>158</v>
+        <v>124</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>81</v>
+        <v>219</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="71" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" s="68" t="s">
-        <v>189</v>
+        <v>63</v>
+      </c>
+      <c r="E26" s="77" t="s">
+        <v>64</v>
+      </c>
+      <c r="F26" s="67" t="s">
+        <v>154</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H26" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H26" s="77" t="s">
+        <v>36</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>159</v>
+        <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" ht="21.9" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>160</v>
+        <v>126</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>85</v>
+        <v>220</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E27" s="66"/>
-      <c r="F27" s="69"/>
+        <v>66</v>
+      </c>
+      <c r="E27" s="70"/>
+      <c r="F27" s="68"/>
       <c r="G27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H27" s="66"/>
+        <v>22</v>
+      </c>
+      <c r="H27" s="70"/>
       <c r="I27" s="31"/>
     </row>
-    <row r="28" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A28" s="8" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>161</v>
+        <v>127</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>88</v>
+        <v>221</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E28" s="67"/>
+        <v>68</v>
+      </c>
+      <c r="E28" s="78"/>
       <c r="F28" s="73"/>
       <c r="G28" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H28" s="67"/>
+        <v>30</v>
+      </c>
+      <c r="H28" s="78"/>
       <c r="I28" s="35" t="s">
-        <v>162</v>
+        <v>128</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="21.9" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>163</v>
+        <v>129</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>91</v>
+        <v>222</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="71" t="s">
-        <v>93</v>
-      </c>
-      <c r="F29" s="68" t="s">
-        <v>190</v>
+        <v>70</v>
+      </c>
+      <c r="E29" s="77" t="s">
+        <v>71</v>
+      </c>
+      <c r="F29" s="67" t="s">
+        <v>155</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H29" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H29" s="77" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="21.9" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>95</v>
+        <v>223</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="E30" s="66"/>
-      <c r="F30" s="69"/>
+        <v>73</v>
+      </c>
+      <c r="E30" s="70"/>
+      <c r="F30" s="68"/>
       <c r="G30" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="H30" s="66"/>
+        <v>132</v>
+      </c>
+      <c r="H30" s="70"/>
       <c r="I30" s="34" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="21.9" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>167</v>
+        <v>133</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E31" s="66"/>
-      <c r="F31" s="69"/>
+        <v>75</v>
+      </c>
+      <c r="E31" s="70"/>
+      <c r="F31" s="68"/>
       <c r="G31" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="H31" s="66"/>
+        <v>134</v>
+      </c>
+      <c r="H31" s="70"/>
       <c r="I31" s="31"/>
     </row>
-    <row r="32" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="21.9" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>170</v>
+        <v>136</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>101</v>
+        <v>225</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E32" s="66"/>
-      <c r="F32" s="69"/>
+        <v>77</v>
+      </c>
+      <c r="E32" s="70"/>
+      <c r="F32" s="68"/>
       <c r="G32" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="H32" s="66"/>
+        <v>137</v>
+      </c>
+      <c r="H32" s="70"/>
       <c r="I32" s="32" t="s">
-        <v>169</v>
+        <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" ht="21.9" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="B33" s="24" t="s">
-        <v>173</v>
+        <v>139</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>104</v>
+        <v>226</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E33" s="66"/>
-      <c r="F33" s="69"/>
+        <v>75</v>
+      </c>
+      <c r="E33" s="70"/>
+      <c r="F33" s="68"/>
       <c r="G33" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="H33" s="66"/>
+        <v>140</v>
+      </c>
+      <c r="H33" s="70"/>
       <c r="I33" s="32" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
       <c r="A34" s="8" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>175</v>
+        <v>141</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>106</v>
+        <v>227</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E34" s="67"/>
-      <c r="F34" s="70"/>
+        <v>77</v>
+      </c>
+      <c r="E34" s="78"/>
+      <c r="F34" s="79"/>
       <c r="G34" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H34" s="67"/>
+        <v>142</v>
+      </c>
+      <c r="H34" s="78"/>
       <c r="I34" s="33"/>
     </row>
-    <row r="35" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" ht="21.9" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>108</v>
+        <v>228</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>191</v>
+        <v>156</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H35" s="71" t="s">
-        <v>49</v>
+        <v>36</v>
+      </c>
+      <c r="H35" s="77" t="s">
+        <v>36</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="N35" s="51"/>
     </row>
-    <row r="36" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>227</v>
+        <v>190</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>112</v>
+        <v>229</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="F36" s="40" t="s">
-        <v>192</v>
+        <v>157</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="67"/>
+        <v>4</v>
+      </c>
+      <c r="H36" s="78"/>
       <c r="I36" s="36" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A37" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E37" s="69" t="s">
+        <v>87</v>
+      </c>
+      <c r="F37" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="G37" s="69" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A38" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>231</v>
+      </c>
+      <c r="D38" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" s="76"/>
+      <c r="F38" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="G38" s="78"/>
+      <c r="H38" s="78"/>
+      <c r="I38" s="38" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A39" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="61" t="s">
+        <v>232</v>
+      </c>
+      <c r="D39" s="64" t="s">
+        <v>233</v>
+      </c>
+      <c r="E39" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="F39" s="42" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="H39" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="I39" s="38" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A40" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="C40" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D40" s="74" t="s">
+        <v>191</v>
+      </c>
+      <c r="E40" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="F40" s="67" t="s">
+        <v>160</v>
+      </c>
+      <c r="G40" s="77" t="s">
+        <v>4</v>
+      </c>
+      <c r="H40" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="I40" s="57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A41" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="B41" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" s="49" t="s">
+        <v>235</v>
+      </c>
+      <c r="D41" s="75"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="73"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="78"/>
+      <c r="I41" s="63" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A42" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" s="48" t="s">
+        <v>186</v>
+      </c>
+      <c r="C42" s="54" t="s">
+        <v>236</v>
+      </c>
+      <c r="D42" s="56" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F42" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="G42" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="H42" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="I42" s="38" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A43" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C43" s="65" t="s">
+        <v>237</v>
+      </c>
+      <c r="D43" s="53" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="65" t="s">
-        <v>117</v>
-      </c>
-      <c r="F37" s="41" t="s">
-        <v>193</v>
-      </c>
-      <c r="G37" s="65" t="s">
-        <v>49</v>
-      </c>
-      <c r="H37" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="I37" s="37" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B38" s="48" t="s">
-        <v>181</v>
-      </c>
-      <c r="C38" s="49" t="s">
-        <v>119</v>
-      </c>
-      <c r="D38" s="50" t="s">
-        <v>120</v>
-      </c>
-      <c r="E38" s="80"/>
-      <c r="F38" s="45" t="s">
-        <v>194</v>
-      </c>
-      <c r="G38" s="67"/>
-      <c r="H38" s="67"/>
-      <c r="I38" s="38" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="C39" s="61" t="s">
-        <v>127</v>
-      </c>
-      <c r="D39" s="64" t="s">
-        <v>184</v>
-      </c>
-      <c r="E39" s="60" t="s">
-        <v>48</v>
-      </c>
-      <c r="F39" s="42" t="s">
-        <v>196</v>
-      </c>
-      <c r="G39" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="H39" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="I39" s="38" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="B40" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="C40" s="43" t="s">
-        <v>122</v>
-      </c>
-      <c r="D40" s="85" t="s">
-        <v>228</v>
-      </c>
-      <c r="E40" s="65" t="s">
-        <v>236</v>
-      </c>
-      <c r="F40" s="68" t="s">
-        <v>195</v>
-      </c>
-      <c r="G40" s="71" t="s">
-        <v>10</v>
-      </c>
-      <c r="H40" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="I40" s="57" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="55" t="s">
-        <v>123</v>
-      </c>
-      <c r="B41" s="48" t="s">
-        <v>185</v>
-      </c>
-      <c r="C41" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="D41" s="86"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="73"/>
-      <c r="G41" s="80"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="63" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="B42" s="48" t="s">
-        <v>222</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>223</v>
-      </c>
-      <c r="D42" s="56" t="s">
-        <v>225</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F42" s="42" t="s">
-        <v>224</v>
-      </c>
-      <c r="G42" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H42" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="I42" s="38" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
-        <v>200</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="C43" s="81" t="s">
-        <v>218</v>
-      </c>
-      <c r="D43" s="53" t="s">
-        <v>213</v>
-      </c>
-      <c r="E43" s="65" t="s">
-        <v>48</v>
-      </c>
-      <c r="F43" s="68" t="s">
-        <v>195</v>
+      <c r="E43" s="69" t="s">
+        <v>35</v>
+      </c>
+      <c r="F43" s="67" t="s">
+        <v>160</v>
       </c>
       <c r="G43" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="H43" s="83" t="s">
-        <v>49</v>
+        <v>22</v>
+      </c>
+      <c r="H43" s="71" t="s">
+        <v>36</v>
       </c>
       <c r="I43" s="47"/>
     </row>
-    <row r="44" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" ht="21.9" customHeight="1">
       <c r="A44" s="11" t="s">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="C44" s="82"/>
+        <v>172</v>
+      </c>
+      <c r="C44" s="66"/>
       <c r="D44" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="E44" s="66"/>
-      <c r="F44" s="69"/>
+        <v>179</v>
+      </c>
+      <c r="E44" s="70"/>
+      <c r="F44" s="68"/>
       <c r="G44" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="H44" s="84"/>
+        <v>30</v>
+      </c>
+      <c r="H44" s="72"/>
       <c r="I44" s="34" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" ht="21.9" customHeight="1">
       <c r="A45" s="11" t="s">
-        <v>203</v>
+        <v>168</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="C45" s="82"/>
+        <v>173</v>
+      </c>
+      <c r="C45" s="66"/>
       <c r="D45" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="E45" s="66"/>
-      <c r="F45" s="69"/>
+        <v>177</v>
+      </c>
+      <c r="E45" s="70"/>
+      <c r="F45" s="68"/>
       <c r="G45" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45" s="84"/>
+        <v>32</v>
+      </c>
+      <c r="H45" s="72"/>
     </row>
-    <row r="46" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" ht="21.9" customHeight="1">
       <c r="A46" s="11" t="s">
-        <v>204</v>
+        <v>169</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="C46" s="82"/>
+        <v>174</v>
+      </c>
+      <c r="C46" s="66"/>
       <c r="D46" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="E46" s="66"/>
-      <c r="F46" s="69"/>
+        <v>180</v>
+      </c>
+      <c r="E46" s="70"/>
+      <c r="F46" s="68"/>
       <c r="G46" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="H46" s="84"/>
+        <v>25</v>
+      </c>
+      <c r="H46" s="72"/>
       <c r="I46" s="57" t="s">
-        <v>220</v>
+        <v>184</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" ht="21.9" customHeight="1">
       <c r="A47" s="11" t="s">
-        <v>205</v>
+        <v>170</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>210</v>
-      </c>
-      <c r="C47" s="82"/>
+        <v>175</v>
+      </c>
+      <c r="C47" s="66"/>
       <c r="D47" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="E47" s="66"/>
-      <c r="F47" s="69"/>
+        <v>181</v>
+      </c>
+      <c r="E47" s="70"/>
+      <c r="F47" s="68"/>
       <c r="G47" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="H47" s="84"/>
+        <v>15</v>
+      </c>
+      <c r="H47" s="72"/>
       <c r="I47" s="52"/>
     </row>
-    <row r="48" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14" ht="21.9" customHeight="1">
       <c r="A48" s="11" t="s">
-        <v>206</v>
+        <v>171</v>
       </c>
       <c r="B48" s="24" t="s">
-        <v>211</v>
-      </c>
-      <c r="C48" s="82"/>
+        <v>176</v>
+      </c>
+      <c r="C48" s="66"/>
       <c r="D48" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="E48" s="66"/>
-      <c r="F48" s="69"/>
+        <v>182</v>
+      </c>
+      <c r="E48" s="70"/>
+      <c r="F48" s="68"/>
       <c r="G48" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="H48" s="84"/>
+        <v>19</v>
+      </c>
+      <c r="H48" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="E2:E11"/>
+    <mergeCell ref="F2:F11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="F12:F20"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="F21:F25"/>
+    <mergeCell ref="H21:H25"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E29:E34"/>
+    <mergeCell ref="F29:F34"/>
+    <mergeCell ref="H29:H34"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="H37:H38"/>
     <mergeCell ref="C43:C48"/>
     <mergeCell ref="F43:F48"/>
     <mergeCell ref="E43:E48"/>
@@ -6088,27 +6034,6 @@
     <mergeCell ref="E40:E41"/>
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
-    <mergeCell ref="E29:E34"/>
-    <mergeCell ref="F29:F34"/>
-    <mergeCell ref="H29:H34"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="H37:H38"/>
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="F21:F25"/>
-    <mergeCell ref="H21:H25"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E2:E11"/>
-    <mergeCell ref="F2:F11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="F12:F20"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="H19:H20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Translate Labs/Other pictures to english (#162)
* feat(APS): add labs, others
</commit_message>
<xml_diff>
--- a/.pic/Labs/lab_05_decoder/rv32i_summary.xlsx
+++ b/.pic/Labs/lab_05_decoder/rv32i_summary.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\voult\Desktop\APS-reborn\.pic\Labs\lab_05_decoder\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA97E5B9-6102-46D4-A302-BF886277C454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{EB09394A-D6B3-4632-AD26-E6834047279C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30936" windowHeight="17496"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,27 +29,9 @@
     <t>Instr</t>
   </si>
   <si>
-    <t>Название</t>
-  </si>
-  <si>
-    <t>Функция</t>
-  </si>
-  <si>
-    <t>Описание</t>
-  </si>
-  <si>
-    <t>Формат</t>
-  </si>
-  <si>
-    <t>Пример использования</t>
-  </si>
-  <si>
     <t>add</t>
   </si>
   <si>
-    <t>Сложение</t>
-  </si>
-  <si>
     <t>rd = rs1 + rs2</t>
   </si>
   <si>
@@ -71,9 +47,6 @@
     <t>sub</t>
   </si>
   <si>
-    <t>Вычитание</t>
-  </si>
-  <si>
     <t>rd = rs1 – rs2</t>
   </si>
   <si>
@@ -116,9 +89,6 @@
     <t>sll</t>
   </si>
   <si>
-    <t>Логический сдвиг влево</t>
-  </si>
-  <si>
     <t>rd = rs1 &lt;&lt; rs2</t>
   </si>
   <si>
@@ -128,9 +98,6 @@
     <t>srl</t>
   </si>
   <si>
-    <t>Логический сдвиг вправо</t>
-  </si>
-  <si>
     <t>rd = rs1 &gt;&gt; rs2</t>
   </si>
   <si>
@@ -140,18 +107,12 @@
     <t>sra</t>
   </si>
   <si>
-    <t>Арифметический сдвиг вправо</t>
-  </si>
-  <si>
     <t>rd = rs1 &gt;&gt;&gt; rs2</t>
   </si>
   <si>
     <t>slt</t>
   </si>
   <si>
-    <t>Результат сравнения A &lt; B</t>
-  </si>
-  <si>
     <t>rd = (rs1 &lt; rs2) ? 1 : 0</t>
   </si>
   <si>
@@ -161,18 +122,12 @@
     <t>sltu</t>
   </si>
   <si>
-    <t>Беззнаковое сравнение A &lt; B</t>
-  </si>
-  <si>
     <t>0x3</t>
   </si>
   <si>
     <t>addi</t>
   </si>
   <si>
-    <t>Сложение с константой</t>
-  </si>
-  <si>
     <t>rd = rs1 + imm</t>
   </si>
   <si>
@@ -230,54 +185,36 @@
     <t>lb</t>
   </si>
   <si>
-    <t>Загрузить байт из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][7:0])</t>
   </si>
   <si>
     <t>lh</t>
   </si>
   <si>
-    <t>Загрузить полуслово из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][15:0])</t>
   </si>
   <si>
     <t>lw</t>
   </si>
   <si>
-    <t>Загрузить слово из памяти</t>
-  </si>
-  <si>
     <t>rd = SE(Mem[rs1 + imm][31:0])</t>
   </si>
   <si>
     <t>lbu</t>
   </si>
   <si>
-    <t>Загрузить беззнаковый байт из памяти</t>
-  </si>
-  <si>
     <t>rd = Mem[rs1 + imm][7:0]</t>
   </si>
   <si>
     <t>lhu</t>
   </si>
   <si>
-    <t>Загрузить беззнаковое полуслово из памяти</t>
-  </si>
-  <si>
     <t>rd = Mem[rs1 + imm][15:0]</t>
   </si>
   <si>
     <t>sb</t>
   </si>
   <si>
-    <t>Сохранить байт в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][7:0] = rs2[7:0]</t>
   </si>
   <si>
@@ -287,27 +224,18 @@
     <t>sh</t>
   </si>
   <si>
-    <t>Сохранить полуслово в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][15:0] = rs2[15:0]</t>
   </si>
   <si>
     <t>sw</t>
   </si>
   <si>
-    <t>Сохранить слово в память</t>
-  </si>
-  <si>
     <t>Mem[rs1 + imm][31:0] = rs2[31:0]</t>
   </si>
   <si>
     <t>beq</t>
   </si>
   <si>
-    <t>Перейти, если A == B</t>
-  </si>
-  <si>
     <t>if (rs1 == rs2) PC += imm</t>
   </si>
   <si>
@@ -317,48 +245,30 @@
     <t>bne</t>
   </si>
   <si>
-    <t>Перейти, если A != B</t>
-  </si>
-  <si>
     <t>if (rs1 != rs2) PC += imm</t>
   </si>
   <si>
     <t>blt</t>
   </si>
   <si>
-    <t>Перейти, если A &lt; B</t>
-  </si>
-  <si>
     <t>if (rs1 &lt; rs2) PC += imm</t>
   </si>
   <si>
     <t>bge</t>
   </si>
   <si>
-    <t>Перейти, если A &gt;= B</t>
-  </si>
-  <si>
     <t>if (rs1 &gt;= rs2) PC += imm</t>
   </si>
   <si>
     <t>bltu</t>
   </si>
   <si>
-    <t>Перейти, если A &lt; B беззнаковое</t>
-  </si>
-  <si>
     <t>bgeu</t>
   </si>
   <si>
-    <t>Перейти, если A &gt;= B беззнаковое</t>
-  </si>
-  <si>
     <t>jal</t>
   </si>
   <si>
-    <t>Переход с сохранением адреса возврата</t>
-  </si>
-  <si>
     <t>rd = PC + 4; PC += imm</t>
   </si>
   <si>
@@ -368,18 +278,12 @@
     <t>jalr</t>
   </si>
   <si>
-    <t>Переход по регистру с сохранением адреса возврата</t>
-  </si>
-  <si>
     <t>rd = PC + 4; PC = rs1 + imm</t>
   </si>
   <si>
     <t>lui</t>
   </si>
   <si>
-    <t>Загрузить константу в сдвинутую на 12</t>
-  </si>
-  <si>
     <t>rd = imm &lt;&lt; 12</t>
   </si>
   <si>
@@ -389,31 +293,19 @@
     <t>auipc</t>
   </si>
   <si>
-    <t>Сохранить счетчик команд в сумме с константой &lt;&lt; 12</t>
-  </si>
-  <si>
     <t>rd = PC + (imm &lt;&lt; 12)</t>
   </si>
   <si>
     <t>ecall</t>
   </si>
   <si>
-    <t>Передача управления операционной системе</t>
-  </si>
-  <si>
     <t>ebreak</t>
   </si>
   <si>
-    <t>Передача управления отладчику</t>
-  </si>
-  <si>
     <t>fence</t>
   </si>
   <si>
     <t>FENCE</t>
-  </si>
-  <si>
-    <t>Синхронизация инструкций с потоками данных</t>
   </si>
   <si>
     <r>
@@ -2616,22 +2508,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Воспринимать как </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cascadia Code SemiBold"/>
-        <family val="3"/>
-        <charset val="204"/>
-      </rPr>
-      <t>nop</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>E</t>
     </r>
     <r>
@@ -3587,58 +3463,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Записать в регистровый файл значение </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">-регистра.
-Обновить значение </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>CS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-регистра в соответствии с вызываемой инструкцией (см. описание).</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">csrop </t>
     </r>
     <r>
@@ -3710,9 +3534,6 @@
     </r>
   </si>
   <si>
-    <t>Возврат управления от обработчика прерывания/исключения</t>
-  </si>
-  <si>
     <t>1110011</t>
   </si>
   <si>
@@ -3867,24 +3688,6 @@
   </si>
   <si>
     <t>illegal_instr = 1</t>
-  </si>
-  <si>
-    <t>Побитовое И</t>
-  </si>
-  <si>
-    <t>Побитовое ИЛИ</t>
-  </si>
-  <si>
-    <t>Побитовое Исключающее ИЛИ</t>
-  </si>
-  <si>
-    <t>Побитовое Исключающее ИЛИ с константой</t>
-  </si>
-  <si>
-    <t>Побитовое ИЛИ с константой</t>
-  </si>
-  <si>
-    <t>Побитовое И с константой</t>
   </si>
   <si>
     <r>
@@ -3947,13 +3750,143 @@
       </rPr>
       <t>**</t>
     </r>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>Usage example</t>
+  </si>
+  <si>
+    <t>Addition</t>
+  </si>
+  <si>
+    <t>Subtraction</t>
+  </si>
+  <si>
+    <t>Bitwise exclusive OR</t>
+  </si>
+  <si>
+    <t>Bitwise OR</t>
+  </si>
+  <si>
+    <t>Bitwise AND</t>
+  </si>
+  <si>
+    <t>Logical left shift</t>
+  </si>
+  <si>
+    <t>Logical right shift</t>
+  </si>
+  <si>
+    <t>Arithmetic right shift</t>
+  </si>
+  <si>
+    <t>Result of comparison A &lt; B</t>
+  </si>
+  <si>
+    <t>Unsigned comparison A &lt; B</t>
+  </si>
+  <si>
+    <t>Addition with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise exclusive OR with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise OR with a constant</t>
+  </si>
+  <si>
+    <t>Bitwise AND with a constant</t>
+  </si>
+  <si>
+    <t>Load byte from memory</t>
+  </si>
+  <si>
+    <t>Load halfword from memory</t>
+  </si>
+  <si>
+    <t>Load word from memory</t>
+  </si>
+  <si>
+    <t>Load unsigned byte from memory</t>
+  </si>
+  <si>
+    <t>Load unsigned halfword from memory</t>
+  </si>
+  <si>
+    <t>Store byte to memory</t>
+  </si>
+  <si>
+    <t>Store halfword to memory</t>
+  </si>
+  <si>
+    <t>Store word to memory</t>
+  </si>
+  <si>
+    <t>Branch if A == B</t>
+  </si>
+  <si>
+    <t>Branch if A != B</t>
+  </si>
+  <si>
+    <t>Branch if A &lt; B</t>
+  </si>
+  <si>
+    <t>Branch if A &gt;= B</t>
+  </si>
+  <si>
+    <t>Branch if A &lt; B, unsigned</t>
+  </si>
+  <si>
+    <t>Branch if A &gt;= B, unsigned</t>
+  </si>
+  <si>
+    <t>Jump saving the return address</t>
+  </si>
+  <si>
+    <t>Register jump saving the return address</t>
+  </si>
+  <si>
+    <t>Load a constant shifted left by 12</t>
+  </si>
+  <si>
+    <t>Save the program counter summed with a constant &lt;&lt; 12</t>
+  </si>
+  <si>
+    <t>Synchronization of instructions with data streams</t>
+  </si>
+  <si>
+    <t>Treat as nop</t>
+  </si>
+  <si>
+    <t>Transfer control to the operating system</t>
+  </si>
+  <si>
+    <t>Transfer control to the debugger</t>
+  </si>
+  <si>
+    <t>Return of control from an interrupt/exception handler</t>
+  </si>
+  <si>
+    <t>Write the value of the CS register to the register file.
+Update the value of the CS register according to the invoked instruction (see description).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4070,14 +4003,6 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color rgb="FF000000"/>
-      <name val="Cascadia Code SemiBold"/>
-      <family val="3"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
       <color rgb="FF4472C4"/>
       <name val="Code Saver"/>
       <family val="3"/>
@@ -4538,34 +4463,55 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4582,27 +4528,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4915,1170 +4840,1191 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4B31E3-B287-4359-8B24-03B2324659CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N48"/>
-  <sheetFormatPr defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="21.9" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="87.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="14.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="87.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I1" s="27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="B2" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="E2" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F2" s="67" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="I1" s="27" t="s">
+      <c r="H2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+    <row r="3" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="B3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="D3" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="E3" s="70"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="65" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="68" t="s">
-        <v>186</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="B4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="E4" s="70"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="H4" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+    <row r="5" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="C5" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="66"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H3" s="2" t="s">
+      <c r="E5" s="70"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="H5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I5" s="30" t="s">
+        <v>95</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
+    <row r="6" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="66"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="2" t="s">
+      <c r="C6" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="E6" s="70"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="66"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="30" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="66"/>
-      <c r="F6" s="69"/>
-      <c r="G6" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I6" s="31"/>
     </row>
-    <row r="7" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="21.9" customHeight="1">
       <c r="A7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="70"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="70"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="32" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="66"/>
-      <c r="F7" s="69"/>
-      <c r="G7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="32" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="66"/>
-      <c r="F8" s="69"/>
-      <c r="G8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" s="32" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="66"/>
-      <c r="F9" s="69"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="68"/>
       <c r="G9" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I9" s="31"/>
     </row>
-    <row r="10" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="21.9" customHeight="1">
       <c r="A10" s="8" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>39</v>
+        <v>208</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="66"/>
-      <c r="F10" s="69"/>
+        <v>29</v>
+      </c>
+      <c r="E10" s="70"/>
+      <c r="F10" s="68"/>
       <c r="G10" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I10" s="31"/>
     </row>
-    <row r="11" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A11" s="8" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>43</v>
+        <v>209</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="67"/>
-      <c r="F11" s="70"/>
+        <v>29</v>
+      </c>
+      <c r="E11" s="78"/>
+      <c r="F11" s="79"/>
       <c r="G11" s="2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I11" s="33"/>
     </row>
-    <row r="12" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="21.9" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>46</v>
+        <v>210</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="72" t="s">
-        <v>187</v>
+        <v>34</v>
+      </c>
+      <c r="E12" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="80" t="s">
+        <v>152</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" s="65" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H12" s="69" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="21.9" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>141</v>
+        <v>107</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>232</v>
+        <v>211</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="66"/>
-      <c r="F13" s="69"/>
+        <v>38</v>
+      </c>
+      <c r="E13" s="70"/>
+      <c r="F13" s="68"/>
       <c r="G13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" s="66"/>
+        <v>11</v>
+      </c>
+      <c r="H13" s="70"/>
       <c r="I13" s="31"/>
     </row>
-    <row r="14" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="21.9" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>142</v>
+        <v>108</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>233</v>
+        <v>212</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="66"/>
-      <c r="F14" s="69"/>
+        <v>40</v>
+      </c>
+      <c r="E14" s="70"/>
+      <c r="F14" s="68"/>
       <c r="G14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="70"/>
+      <c r="I14" s="34" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A15" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="70"/>
+      <c r="F15" s="68"/>
+      <c r="G15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="70"/>
+    </row>
+    <row r="16" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A16" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="81" t="s">
+        <v>192</v>
+      </c>
+      <c r="F16" s="68"/>
+      <c r="G16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="66"/>
-      <c r="I14" s="34" t="s">
-        <v>140</v>
+      <c r="H16" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="66"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="66"/>
+    <row r="17" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A17" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="82"/>
+      <c r="F17" s="68"/>
+      <c r="G17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I17" s="32" t="s">
+        <v>111</v>
+      </c>
     </row>
-    <row r="16" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E16" s="74" t="s">
-        <v>235</v>
-      </c>
-      <c r="F16" s="69"/>
-      <c r="G16" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" s="32" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="75"/>
-      <c r="F17" s="69"/>
-      <c r="G17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" s="32" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="21.9" customHeight="1">
       <c r="A18" s="22" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>148</v>
+        <v>114</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>36</v>
+        <v>207</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="E18" s="76"/>
-      <c r="F18" s="69"/>
+        <v>48</v>
+      </c>
+      <c r="E18" s="83"/>
+      <c r="F18" s="68"/>
       <c r="G18" s="5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I18" s="31"/>
     </row>
-    <row r="19" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="21.9" customHeight="1">
       <c r="A19" s="8" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>149</v>
+        <v>115</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>39</v>
+        <v>208</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="F19" s="69"/>
+        <v>50</v>
+      </c>
+      <c r="E19" s="84" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="68"/>
       <c r="G19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H19" s="79" t="s">
-        <v>49</v>
+        <v>30</v>
+      </c>
+      <c r="H19" s="86" t="s">
+        <v>36</v>
       </c>
       <c r="I19" s="31"/>
     </row>
-    <row r="20" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A20" s="8" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>43</v>
+        <v>209</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="78"/>
+        <v>50</v>
+      </c>
+      <c r="E20" s="85"/>
       <c r="F20" s="73"/>
       <c r="G20" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" s="67"/>
+        <v>32</v>
+      </c>
+      <c r="H20" s="78"/>
       <c r="I20" s="33"/>
     </row>
-    <row r="21" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="21.9" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>66</v>
+        <v>214</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="F21" s="68" t="s">
-        <v>188</v>
+        <v>53</v>
+      </c>
+      <c r="E21" s="77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="67" t="s">
+        <v>153</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H21" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H21" s="77" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="21.9" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>153</v>
+        <v>119</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>69</v>
+        <v>215</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="66"/>
-      <c r="F22" s="69"/>
+        <v>55</v>
+      </c>
+      <c r="E22" s="70"/>
+      <c r="F22" s="68"/>
       <c r="G22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="70"/>
+      <c r="I22" s="34" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="21.9" customHeight="1">
+      <c r="A23" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="70"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H22" s="66"/>
-      <c r="I22" s="34" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>154</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="66"/>
-      <c r="F23" s="69"/>
-      <c r="G23" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H23" s="66"/>
+      <c r="H23" s="70"/>
       <c r="I23" s="31"/>
     </row>
-    <row r="24" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="21.9" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>156</v>
+        <v>122</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>75</v>
+        <v>217</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="E24" s="66"/>
-      <c r="F24" s="69"/>
+        <v>59</v>
+      </c>
+      <c r="E24" s="70"/>
+      <c r="F24" s="68"/>
       <c r="G24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H24" s="66"/>
+        <v>11</v>
+      </c>
+      <c r="H24" s="70"/>
       <c r="I24" s="32" t="s">
-        <v>155</v>
+        <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A25" s="8" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>157</v>
+        <v>123</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>78</v>
+        <v>218</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E25" s="67"/>
+        <v>61</v>
+      </c>
+      <c r="E25" s="78"/>
       <c r="F25" s="73"/>
       <c r="G25" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H25" s="67"/>
+        <v>25</v>
+      </c>
+      <c r="H25" s="78"/>
       <c r="I25" s="33"/>
     </row>
-    <row r="26" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" ht="21.9" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="B26" s="25" t="s">
-        <v>158</v>
+        <v>124</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>81</v>
+        <v>219</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="71" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" s="68" t="s">
-        <v>189</v>
+        <v>63</v>
+      </c>
+      <c r="E26" s="77" t="s">
+        <v>64</v>
+      </c>
+      <c r="F26" s="67" t="s">
+        <v>154</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H26" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H26" s="77" t="s">
+        <v>36</v>
       </c>
       <c r="I26" s="34" t="s">
-        <v>159</v>
+        <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" ht="21.9" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>160</v>
+        <v>126</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>85</v>
+        <v>220</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E27" s="66"/>
-      <c r="F27" s="69"/>
+        <v>66</v>
+      </c>
+      <c r="E27" s="70"/>
+      <c r="F27" s="68"/>
       <c r="G27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H27" s="66"/>
+        <v>22</v>
+      </c>
+      <c r="H27" s="70"/>
       <c r="I27" s="31"/>
     </row>
-    <row r="28" spans="1:9" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" ht="21.9" customHeight="1" thickBot="1">
       <c r="A28" s="8" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>161</v>
+        <v>127</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>88</v>
+        <v>221</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E28" s="67"/>
+        <v>68</v>
+      </c>
+      <c r="E28" s="78"/>
       <c r="F28" s="73"/>
       <c r="G28" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H28" s="67"/>
+        <v>30</v>
+      </c>
+      <c r="H28" s="78"/>
       <c r="I28" s="35" t="s">
-        <v>162</v>
+        <v>128</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="21.9" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>163</v>
+        <v>129</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>91</v>
+        <v>222</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="71" t="s">
-        <v>93</v>
-      </c>
-      <c r="F29" s="68" t="s">
-        <v>190</v>
+        <v>70</v>
+      </c>
+      <c r="E29" s="77" t="s">
+        <v>71</v>
+      </c>
+      <c r="F29" s="67" t="s">
+        <v>155</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H29" s="71" t="s">
-        <v>49</v>
+        <v>4</v>
+      </c>
+      <c r="H29" s="77" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="21.9" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>94</v>
+        <v>72</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>95</v>
+        <v>223</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="E30" s="66"/>
-      <c r="F30" s="69"/>
+        <v>73</v>
+      </c>
+      <c r="E30" s="70"/>
+      <c r="F30" s="68"/>
       <c r="G30" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="H30" s="66"/>
+        <v>132</v>
+      </c>
+      <c r="H30" s="70"/>
       <c r="I30" s="34" t="s">
-        <v>164</v>
+        <v>130</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="21.9" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>167</v>
+        <v>133</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E31" s="66"/>
-      <c r="F31" s="69"/>
+        <v>75</v>
+      </c>
+      <c r="E31" s="70"/>
+      <c r="F31" s="68"/>
       <c r="G31" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="H31" s="66"/>
+        <v>134</v>
+      </c>
+      <c r="H31" s="70"/>
       <c r="I31" s="31"/>
     </row>
-    <row r="32" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="21.9" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>170</v>
+        <v>136</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>101</v>
+        <v>225</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E32" s="66"/>
-      <c r="F32" s="69"/>
+        <v>77</v>
+      </c>
+      <c r="E32" s="70"/>
+      <c r="F32" s="68"/>
       <c r="G32" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="H32" s="66"/>
+        <v>137</v>
+      </c>
+      <c r="H32" s="70"/>
       <c r="I32" s="32" t="s">
-        <v>169</v>
+        <v>135</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" ht="21.9" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="B33" s="24" t="s">
-        <v>173</v>
+        <v>139</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>104</v>
+        <v>226</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E33" s="66"/>
-      <c r="F33" s="69"/>
+        <v>75</v>
+      </c>
+      <c r="E33" s="70"/>
+      <c r="F33" s="68"/>
       <c r="G33" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="H33" s="66"/>
+        <v>140</v>
+      </c>
+      <c r="H33" s="70"/>
       <c r="I33" s="32" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
       <c r="A34" s="8" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>175</v>
+        <v>141</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>106</v>
+        <v>227</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E34" s="67"/>
-      <c r="F34" s="70"/>
+        <v>77</v>
+      </c>
+      <c r="E34" s="78"/>
+      <c r="F34" s="79"/>
       <c r="G34" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H34" s="67"/>
+        <v>142</v>
+      </c>
+      <c r="H34" s="78"/>
       <c r="I34" s="33"/>
     </row>
-    <row r="35" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" ht="21.9" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="B35" s="25" t="s">
-        <v>226</v>
+        <v>189</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>108</v>
+        <v>228</v>
       </c>
       <c r="D35" s="16" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>191</v>
+        <v>156</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H35" s="71" t="s">
-        <v>49</v>
+        <v>36</v>
+      </c>
+      <c r="H35" s="77" t="s">
+        <v>36</v>
       </c>
       <c r="I35" s="36" t="s">
-        <v>177</v>
+        <v>143</v>
       </c>
       <c r="N35" s="51"/>
     </row>
-    <row r="36" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="s">
-        <v>111</v>
+        <v>83</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>227</v>
+        <v>190</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>112</v>
+        <v>229</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="F36" s="40" t="s">
-        <v>192</v>
+        <v>157</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="67"/>
+        <v>4</v>
+      </c>
+      <c r="H36" s="78"/>
       <c r="I36" s="36" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A37" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="D37" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E37" s="69" t="s">
+        <v>87</v>
+      </c>
+      <c r="F37" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="G37" s="69" t="s">
+        <v>36</v>
+      </c>
+      <c r="H37" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" s="37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A38" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="48" t="s">
+        <v>147</v>
+      </c>
+      <c r="C38" s="49" t="s">
+        <v>231</v>
+      </c>
+      <c r="D38" s="50" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" s="76"/>
+      <c r="F38" s="45" t="s">
+        <v>159</v>
+      </c>
+      <c r="G38" s="78"/>
+      <c r="H38" s="78"/>
+      <c r="I38" s="38" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A39" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="61" t="s">
+        <v>232</v>
+      </c>
+      <c r="D39" s="64" t="s">
+        <v>233</v>
+      </c>
+      <c r="E39" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="F39" s="42" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="58" t="s">
+        <v>4</v>
+      </c>
+      <c r="H39" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="I39" s="38" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A40" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="C40" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D40" s="74" t="s">
+        <v>191</v>
+      </c>
+      <c r="E40" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="F40" s="67" t="s">
+        <v>160</v>
+      </c>
+      <c r="G40" s="77" t="s">
+        <v>4</v>
+      </c>
+      <c r="H40" s="77" t="s">
+        <v>36</v>
+      </c>
+      <c r="I40" s="57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A41" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="B41" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" s="49" t="s">
+        <v>235</v>
+      </c>
+      <c r="D41" s="75"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="73"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="78"/>
+      <c r="I41" s="63" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="21.9" customHeight="1" thickBot="1">
+      <c r="A42" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" s="48" t="s">
+        <v>186</v>
+      </c>
+      <c r="C42" s="54" t="s">
+        <v>236</v>
+      </c>
+      <c r="D42" s="56" t="s">
+        <v>188</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F42" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="G42" s="44" t="s">
+        <v>4</v>
+      </c>
+      <c r="H42" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="I42" s="38" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="21.9" customHeight="1">
+      <c r="A43" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="C43" s="65" t="s">
+        <v>237</v>
+      </c>
+      <c r="D43" s="53" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="65" t="s">
-        <v>117</v>
-      </c>
-      <c r="F37" s="41" t="s">
-        <v>193</v>
-      </c>
-      <c r="G37" s="65" t="s">
-        <v>49</v>
-      </c>
-      <c r="H37" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="I37" s="37" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B38" s="48" t="s">
-        <v>181</v>
-      </c>
-      <c r="C38" s="49" t="s">
-        <v>119</v>
-      </c>
-      <c r="D38" s="50" t="s">
-        <v>120</v>
-      </c>
-      <c r="E38" s="80"/>
-      <c r="F38" s="45" t="s">
-        <v>194</v>
-      </c>
-      <c r="G38" s="67"/>
-      <c r="H38" s="67"/>
-      <c r="I38" s="38" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="62" t="s">
-        <v>125</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="C39" s="61" t="s">
-        <v>127</v>
-      </c>
-      <c r="D39" s="64" t="s">
-        <v>184</v>
-      </c>
-      <c r="E39" s="60" t="s">
-        <v>48</v>
-      </c>
-      <c r="F39" s="42" t="s">
-        <v>196</v>
-      </c>
-      <c r="G39" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="H39" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="I39" s="38" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="B40" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="C40" s="43" t="s">
-        <v>122</v>
-      </c>
-      <c r="D40" s="85" t="s">
-        <v>228</v>
-      </c>
-      <c r="E40" s="65" t="s">
-        <v>236</v>
-      </c>
-      <c r="F40" s="68" t="s">
-        <v>195</v>
-      </c>
-      <c r="G40" s="71" t="s">
-        <v>10</v>
-      </c>
-      <c r="H40" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="I40" s="57" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="55" t="s">
-        <v>123</v>
-      </c>
-      <c r="B41" s="48" t="s">
-        <v>185</v>
-      </c>
-      <c r="C41" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="D41" s="86"/>
-      <c r="E41" s="80"/>
-      <c r="F41" s="73"/>
-      <c r="G41" s="80"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="63" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A42" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="B42" s="48" t="s">
-        <v>222</v>
-      </c>
-      <c r="C42" s="54" t="s">
-        <v>223</v>
-      </c>
-      <c r="D42" s="56" t="s">
-        <v>225</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F42" s="42" t="s">
-        <v>224</v>
-      </c>
-      <c r="G42" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H42" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="I42" s="38" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
-        <v>200</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="C43" s="81" t="s">
-        <v>218</v>
-      </c>
-      <c r="D43" s="53" t="s">
-        <v>213</v>
-      </c>
-      <c r="E43" s="65" t="s">
-        <v>48</v>
-      </c>
-      <c r="F43" s="68" t="s">
-        <v>195</v>
+      <c r="E43" s="69" t="s">
+        <v>35</v>
+      </c>
+      <c r="F43" s="67" t="s">
+        <v>160</v>
       </c>
       <c r="G43" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="H43" s="83" t="s">
-        <v>49</v>
+        <v>22</v>
+      </c>
+      <c r="H43" s="71" t="s">
+        <v>36</v>
       </c>
       <c r="I43" s="47"/>
     </row>
-    <row r="44" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" ht="21.9" customHeight="1">
       <c r="A44" s="11" t="s">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="C44" s="82"/>
+        <v>172</v>
+      </c>
+      <c r="C44" s="66"/>
       <c r="D44" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="E44" s="66"/>
-      <c r="F44" s="69"/>
+        <v>179</v>
+      </c>
+      <c r="E44" s="70"/>
+      <c r="F44" s="68"/>
       <c r="G44" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="H44" s="84"/>
+        <v>30</v>
+      </c>
+      <c r="H44" s="72"/>
       <c r="I44" s="34" t="s">
-        <v>219</v>
+        <v>183</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" ht="21.9" customHeight="1">
       <c r="A45" s="11" t="s">
-        <v>203</v>
+        <v>168</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="C45" s="82"/>
+        <v>173</v>
+      </c>
+      <c r="C45" s="66"/>
       <c r="D45" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="E45" s="66"/>
-      <c r="F45" s="69"/>
+        <v>177</v>
+      </c>
+      <c r="E45" s="70"/>
+      <c r="F45" s="68"/>
       <c r="G45" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45" s="84"/>
+        <v>32</v>
+      </c>
+      <c r="H45" s="72"/>
     </row>
-    <row r="46" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" ht="21.9" customHeight="1">
       <c r="A46" s="11" t="s">
-        <v>204</v>
+        <v>169</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="C46" s="82"/>
+        <v>174</v>
+      </c>
+      <c r="C46" s="66"/>
       <c r="D46" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="E46" s="66"/>
-      <c r="F46" s="69"/>
+        <v>180</v>
+      </c>
+      <c r="E46" s="70"/>
+      <c r="F46" s="68"/>
       <c r="G46" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="H46" s="84"/>
+        <v>25</v>
+      </c>
+      <c r="H46" s="72"/>
       <c r="I46" s="57" t="s">
-        <v>220</v>
+        <v>184</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" ht="21.9" customHeight="1">
       <c r="A47" s="11" t="s">
-        <v>205</v>
+        <v>170</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>210</v>
-      </c>
-      <c r="C47" s="82"/>
+        <v>175</v>
+      </c>
+      <c r="C47" s="66"/>
       <c r="D47" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="E47" s="66"/>
-      <c r="F47" s="69"/>
+        <v>181</v>
+      </c>
+      <c r="E47" s="70"/>
+      <c r="F47" s="68"/>
       <c r="G47" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="H47" s="84"/>
+        <v>15</v>
+      </c>
+      <c r="H47" s="72"/>
       <c r="I47" s="52"/>
     </row>
-    <row r="48" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14" ht="21.9" customHeight="1">
       <c r="A48" s="11" t="s">
-        <v>206</v>
+        <v>171</v>
       </c>
       <c r="B48" s="24" t="s">
-        <v>211</v>
-      </c>
-      <c r="C48" s="82"/>
+        <v>176</v>
+      </c>
+      <c r="C48" s="66"/>
       <c r="D48" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="E48" s="66"/>
-      <c r="F48" s="69"/>
+        <v>182</v>
+      </c>
+      <c r="E48" s="70"/>
+      <c r="F48" s="68"/>
       <c r="G48" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="H48" s="84"/>
+        <v>19</v>
+      </c>
+      <c r="H48" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="E2:E11"/>
+    <mergeCell ref="F2:F11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="F12:F20"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="F21:F25"/>
+    <mergeCell ref="H21:H25"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E29:E34"/>
+    <mergeCell ref="F29:F34"/>
+    <mergeCell ref="H29:H34"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="H37:H38"/>
     <mergeCell ref="C43:C48"/>
     <mergeCell ref="F43:F48"/>
     <mergeCell ref="E43:E48"/>
@@ -6088,27 +6034,6 @@
     <mergeCell ref="E40:E41"/>
     <mergeCell ref="G40:G41"/>
     <mergeCell ref="H40:H41"/>
-    <mergeCell ref="E29:E34"/>
-    <mergeCell ref="F29:F34"/>
-    <mergeCell ref="H29:H34"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="H37:H38"/>
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="F21:F25"/>
-    <mergeCell ref="H21:H25"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E2:E11"/>
-    <mergeCell ref="F2:F11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="F12:F20"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="H19:H20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>